<commit_message>
updating model run and metrics scripts
</commit_message>
<xml_diff>
--- a/Runs-description.xlsx
+++ b/Runs-description.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matteoperini/Library/CloudStorage/Box-Box/Matteo Perini/13_NA-returns/Model/NA_SEIR-EAKF_forecast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04FC6208-2289-8347-9758-6FBD22155D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9CB8527-BEFF-3742-956F-9D6217A0890C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4680" yWindow="1640" windowWidth="33720" windowHeight="18180" xr2:uid="{DA942B41-D09C-4741-975D-803349827F2C}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$430</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$430</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1297" uniqueCount="484">
   <si>
     <t>nickname</t>
   </si>
@@ -1048,12 +1048,6 @@
   </si>
   <si>
     <t>tr00</t>
-  </si>
-  <si>
-    <t>Stochastic</t>
-  </si>
-  <si>
-    <t>y</t>
   </si>
   <si>
     <t>601</t>
@@ -1889,8 +1883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67D76F6C-B8F9-3044-BD3D-2174C4F373AB}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:J289"/>
+  <dimension ref="A1:I285"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="2" width="8.83203125" style="1" bestFit="1" customWidth="1"/>
@@ -1901,14 +1894,13 @@
     <col min="7" max="7" width="23.6640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="27.1640625" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.83203125" style="1"/>
+    <col min="10" max="10" width="29.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.33203125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="27.1640625" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -1936,11 +1928,8 @@
       <c r="I1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
         <v>194</v>
       </c>
@@ -1948,7 +1937,7 @@
         <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>76</v>
@@ -1968,11 +1957,8 @@
       <c r="I2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A3" s="1" t="s">
         <v>195</v>
       </c>
@@ -1980,7 +1966,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>77</v>
@@ -2000,11 +1986,8 @@
       <c r="I3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A4" s="1" t="s">
         <v>196</v>
       </c>
@@ -2012,7 +1995,7 @@
         <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>78</v>
@@ -2032,11 +2015,8 @@
       <c r="I4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A5" s="1" t="s">
         <v>197</v>
       </c>
@@ -2044,7 +2024,7 @@
         <v>23</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>79</v>
@@ -2064,11 +2044,8 @@
       <c r="I5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A6" s="1" t="s">
         <v>198</v>
       </c>
@@ -2076,7 +2053,7 @@
         <v>24</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>80</v>
@@ -2096,11 +2073,8 @@
       <c r="I6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A7" s="1" t="s">
         <v>199</v>
       </c>
@@ -2108,7 +2082,7 @@
         <v>25</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>81</v>
@@ -2128,11 +2102,8 @@
       <c r="I7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A8" s="1" t="s">
         <v>200</v>
       </c>
@@ -2140,7 +2111,7 @@
         <v>26</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>82</v>
@@ -2160,11 +2131,8 @@
       <c r="I8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A9" s="1" t="s">
         <v>201</v>
       </c>
@@ -2172,7 +2140,7 @@
         <v>27</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>83</v>
@@ -2192,11 +2160,8 @@
       <c r="I9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A10" s="1" t="s">
         <v>202</v>
       </c>
@@ -2204,7 +2169,7 @@
         <v>28</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>84</v>
@@ -2224,11 +2189,8 @@
       <c r="I10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A11" s="1" t="s">
         <v>203</v>
       </c>
@@ -2236,7 +2198,7 @@
         <v>29</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>85</v>
@@ -2256,11 +2218,8 @@
       <c r="I11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A12" s="1" t="s">
         <v>204</v>
       </c>
@@ -2268,7 +2227,7 @@
         <v>30</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>86</v>
@@ -2288,11 +2247,8 @@
       <c r="I12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A13" s="1" t="s">
         <v>205</v>
       </c>
@@ -2300,7 +2256,7 @@
         <v>31</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>87</v>
@@ -2320,11 +2276,8 @@
       <c r="I13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J13" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A14" s="1" t="s">
         <v>206</v>
       </c>
@@ -2332,7 +2285,7 @@
         <v>32</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>88</v>
@@ -2352,11 +2305,8 @@
       <c r="I14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A15" s="1" t="s">
         <v>207</v>
       </c>
@@ -2364,7 +2314,7 @@
         <v>33</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>89</v>
@@ -2384,11 +2334,8 @@
       <c r="I15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A16" s="1" t="s">
         <v>208</v>
       </c>
@@ -2396,7 +2343,7 @@
         <v>34</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>90</v>
@@ -2416,11 +2363,8 @@
       <c r="I16" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J16" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A17" s="1" t="s">
         <v>209</v>
       </c>
@@ -2428,7 +2372,7 @@
         <v>35</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>91</v>
@@ -2448,11 +2392,8 @@
       <c r="I17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A18" s="1" t="s">
         <v>210</v>
       </c>
@@ -2460,7 +2401,7 @@
         <v>36</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>92</v>
@@ -2480,11 +2421,8 @@
       <c r="I18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A19" s="1" t="s">
         <v>211</v>
       </c>
@@ -2492,7 +2430,7 @@
         <v>37</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>93</v>
@@ -2512,11 +2450,8 @@
       <c r="I19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A20" s="1" t="s">
         <v>212</v>
       </c>
@@ -2524,7 +2459,7 @@
         <v>38</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>94</v>
@@ -2544,11 +2479,8 @@
       <c r="I20" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A21" s="1" t="s">
         <v>213</v>
       </c>
@@ -2556,7 +2488,7 @@
         <v>39</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>95</v>
@@ -2576,11 +2508,8 @@
       <c r="I21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A22" s="1" t="s">
         <v>214</v>
       </c>
@@ -2588,7 +2517,7 @@
         <v>40</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>96</v>
@@ -2608,11 +2537,8 @@
       <c r="I22" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A23" s="1" t="s">
         <v>215</v>
       </c>
@@ -2620,7 +2546,7 @@
         <v>41</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>97</v>
@@ -2640,11 +2566,8 @@
       <c r="I23" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J23" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A24" s="1" t="s">
         <v>216</v>
       </c>
@@ -2652,7 +2575,7 @@
         <v>42</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>98</v>
@@ -2672,11 +2595,8 @@
       <c r="I24" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J24" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A25" s="1" t="s">
         <v>217</v>
       </c>
@@ -2684,7 +2604,7 @@
         <v>43</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>99</v>
@@ -2704,11 +2624,8 @@
       <c r="I25" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A26" s="1" t="s">
         <v>218</v>
       </c>
@@ -2716,7 +2633,7 @@
         <v>44</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>100</v>
@@ -2736,11 +2653,8 @@
       <c r="I26" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J26" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A27" s="1" t="s">
         <v>219</v>
       </c>
@@ -2748,7 +2662,7 @@
         <v>45</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>101</v>
@@ -2768,11 +2682,8 @@
       <c r="I27" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A28" s="1" t="s">
         <v>220</v>
       </c>
@@ -2780,7 +2691,7 @@
         <v>46</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>102</v>
@@ -2800,11 +2711,8 @@
       <c r="I28" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J28" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A29" s="1" t="s">
         <v>221</v>
       </c>
@@ -2812,7 +2720,7 @@
         <v>47</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>103</v>
@@ -2832,11 +2740,8 @@
       <c r="I29" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J29" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A30" s="1" t="s">
         <v>222</v>
       </c>
@@ -2844,7 +2749,7 @@
         <v>48</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>104</v>
@@ -2864,11 +2769,8 @@
       <c r="I30" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A31" s="1" t="s">
         <v>223</v>
       </c>
@@ -2876,7 +2778,7 @@
         <v>49</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>105</v>
@@ -2896,11 +2798,8 @@
       <c r="I31" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A32" s="1" t="s">
         <v>224</v>
       </c>
@@ -2908,7 +2807,7 @@
         <v>50</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>106</v>
@@ -2928,11 +2827,8 @@
       <c r="I32" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J32" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A33" s="1" t="s">
         <v>225</v>
       </c>
@@ -2940,7 +2836,7 @@
         <v>51</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>107</v>
@@ -2960,11 +2856,8 @@
       <c r="I33" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J33" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A34" s="1" t="s">
         <v>226</v>
       </c>
@@ -2972,7 +2865,7 @@
         <v>52</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>108</v>
@@ -2992,11 +2885,8 @@
       <c r="I34" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J34" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A35" s="1" t="s">
         <v>227</v>
       </c>
@@ -3004,7 +2894,7 @@
         <v>53</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>109</v>
@@ -3024,11 +2914,8 @@
       <c r="I35" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J35" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A36" s="1" t="s">
         <v>228</v>
       </c>
@@ -3036,7 +2923,7 @@
         <v>54</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>110</v>
@@ -3056,11 +2943,8 @@
       <c r="I36" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J36" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A37" s="1" t="s">
         <v>229</v>
       </c>
@@ -3068,7 +2952,7 @@
         <v>55</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>76</v>
@@ -3088,11 +2972,8 @@
       <c r="I37" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J37" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A38" s="1" t="s">
         <v>230</v>
       </c>
@@ -3100,7 +2981,7 @@
         <v>56</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>77</v>
@@ -3120,11 +3001,8 @@
       <c r="I38" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J38" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A39" s="1" t="s">
         <v>231</v>
       </c>
@@ -3132,7 +3010,7 @@
         <v>57</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>78</v>
@@ -3152,11 +3030,8 @@
       <c r="I39" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J39" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A40" s="1" t="s">
         <v>232</v>
       </c>
@@ -3164,7 +3039,7 @@
         <v>58</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>79</v>
@@ -3184,11 +3059,8 @@
       <c r="I40" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J40" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A41" s="1" t="s">
         <v>233</v>
       </c>
@@ -3196,7 +3068,7 @@
         <v>59</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>80</v>
@@ -3216,11 +3088,8 @@
       <c r="I41" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J41" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A42" s="1" t="s">
         <v>234</v>
       </c>
@@ -3228,7 +3097,7 @@
         <v>60</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>81</v>
@@ -3248,11 +3117,8 @@
       <c r="I42" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J42" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A43" s="1" t="s">
         <v>235</v>
       </c>
@@ -3260,7 +3126,7 @@
         <v>61</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>82</v>
@@ -3280,11 +3146,8 @@
       <c r="I43" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J43" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A44" s="1" t="s">
         <v>236</v>
       </c>
@@ -3292,7 +3155,7 @@
         <v>62</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>83</v>
@@ -3312,11 +3175,8 @@
       <c r="I44" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J44" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A45" s="1" t="s">
         <v>237</v>
       </c>
@@ -3324,7 +3184,7 @@
         <v>63</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>84</v>
@@ -3344,11 +3204,8 @@
       <c r="I45" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J45" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A46" s="1" t="s">
         <v>238</v>
       </c>
@@ -3356,7 +3213,7 @@
         <v>64</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>85</v>
@@ -3376,11 +3233,8 @@
       <c r="I46" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J46" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A47" s="1" t="s">
         <v>239</v>
       </c>
@@ -3388,7 +3242,7 @@
         <v>65</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>86</v>
@@ -3408,11 +3262,8 @@
       <c r="I47" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J47" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A48" s="1" t="s">
         <v>240</v>
       </c>
@@ -3420,7 +3271,7 @@
         <v>66</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>87</v>
@@ -3440,11 +3291,8 @@
       <c r="I48" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J48" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A49" s="1" t="s">
         <v>241</v>
       </c>
@@ -3452,7 +3300,7 @@
         <v>67</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>88</v>
@@ -3472,11 +3320,8 @@
       <c r="I49" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J49" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A50" s="1" t="s">
         <v>242</v>
       </c>
@@ -3484,7 +3329,7 @@
         <v>68</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>89</v>
@@ -3504,11 +3349,8 @@
       <c r="I50" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J50" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A51" s="1" t="s">
         <v>243</v>
       </c>
@@ -3516,7 +3358,7 @@
         <v>69</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>90</v>
@@ -3536,11 +3378,8 @@
       <c r="I51" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J51" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A52" s="1" t="s">
         <v>244</v>
       </c>
@@ -3548,7 +3387,7 @@
         <v>70</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>91</v>
@@ -3568,11 +3407,8 @@
       <c r="I52" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J52" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A53" s="1" t="s">
         <v>245</v>
       </c>
@@ -3580,7 +3416,7 @@
         <v>71</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>92</v>
@@ -3600,11 +3436,8 @@
       <c r="I53" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J53" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A54" s="1" t="s">
         <v>246</v>
       </c>
@@ -3612,7 +3445,7 @@
         <v>72</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>93</v>
@@ -3632,11 +3465,8 @@
       <c r="I54" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J54" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A55" s="1" t="s">
         <v>247</v>
       </c>
@@ -3644,7 +3474,7 @@
         <v>73</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>94</v>
@@ -3664,11 +3494,8 @@
       <c r="I55" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J55" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A56" s="1" t="s">
         <v>248</v>
       </c>
@@ -3676,7 +3503,7 @@
         <v>74</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>95</v>
@@ -3696,11 +3523,8 @@
       <c r="I56" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J56" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A57" s="1" t="s">
         <v>249</v>
       </c>
@@ -3708,7 +3532,7 @@
         <v>75</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>96</v>
@@ -3728,11 +3552,8 @@
       <c r="I57" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J57" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A58" s="1" t="s">
         <v>250</v>
       </c>
@@ -3740,7 +3561,7 @@
         <v>151</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>97</v>
@@ -3760,11 +3581,8 @@
       <c r="I58" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J58" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A59" s="1" t="s">
         <v>251</v>
       </c>
@@ -3772,7 +3590,7 @@
         <v>152</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>98</v>
@@ -3792,11 +3610,8 @@
       <c r="I59" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J59" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A60" s="1" t="s">
         <v>252</v>
       </c>
@@ -3804,7 +3619,7 @@
         <v>153</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>99</v>
@@ -3824,11 +3639,8 @@
       <c r="I60" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J60" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A61" s="1" t="s">
         <v>253</v>
       </c>
@@ -3836,7 +3648,7 @@
         <v>154</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>100</v>
@@ -3856,11 +3668,8 @@
       <c r="I61" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J61" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A62" s="1" t="s">
         <v>254</v>
       </c>
@@ -3868,7 +3677,7 @@
         <v>155</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>101</v>
@@ -3888,11 +3697,8 @@
       <c r="I62" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J62" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A63" s="1" t="s">
         <v>255</v>
       </c>
@@ -3900,7 +3706,7 @@
         <v>156</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>102</v>
@@ -3920,11 +3726,8 @@
       <c r="I63" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J63" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A64" s="1" t="s">
         <v>256</v>
       </c>
@@ -3932,7 +3735,7 @@
         <v>157</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>103</v>
@@ -3952,11 +3755,8 @@
       <c r="I64" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J64" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A65" s="1" t="s">
         <v>257</v>
       </c>
@@ -3964,7 +3764,7 @@
         <v>158</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>104</v>
@@ -3984,11 +3784,8 @@
       <c r="I65" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J65" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A66" s="1" t="s">
         <v>258</v>
       </c>
@@ -3996,7 +3793,7 @@
         <v>159</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="D66" s="1" t="s">
         <v>105</v>
@@ -4016,11 +3813,8 @@
       <c r="I66" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J66" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A67" s="1" t="s">
         <v>259</v>
       </c>
@@ -4028,7 +3822,7 @@
         <v>160</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="D67" s="1" t="s">
         <v>106</v>
@@ -4048,11 +3842,8 @@
       <c r="I67" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J67" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A68" s="1" t="s">
         <v>260</v>
       </c>
@@ -4060,7 +3851,7 @@
         <v>161</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>107</v>
@@ -4080,11 +3871,8 @@
       <c r="I68" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J68" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A69" s="1" t="s">
         <v>261</v>
       </c>
@@ -4092,7 +3880,7 @@
         <v>162</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>108</v>
@@ -4112,11 +3900,8 @@
       <c r="I69" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J69" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A70" s="1" t="s">
         <v>262</v>
       </c>
@@ -4124,7 +3909,7 @@
         <v>163</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>109</v>
@@ -4144,11 +3929,8 @@
       <c r="I70" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J70" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A71" s="1" t="s">
         <v>263</v>
       </c>
@@ -4156,7 +3938,7 @@
         <v>164</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="D71" s="1" t="s">
         <v>110</v>
@@ -4176,11 +3958,8 @@
       <c r="I71" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J71" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A72" s="1" t="s">
         <v>264</v>
       </c>
@@ -4188,7 +3967,7 @@
         <v>165</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D72" s="1" t="s">
         <v>76</v>
@@ -4208,11 +3987,8 @@
       <c r="I72" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J72" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A73" s="1" t="s">
         <v>265</v>
       </c>
@@ -4220,7 +3996,7 @@
         <v>166</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>77</v>
@@ -4240,11 +4016,8 @@
       <c r="I73" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J73" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A74" s="1" t="s">
         <v>266</v>
       </c>
@@ -4252,7 +4025,7 @@
         <v>167</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>78</v>
@@ -4272,11 +4045,8 @@
       <c r="I74" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J74" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A75" s="1" t="s">
         <v>267</v>
       </c>
@@ -4284,7 +4054,7 @@
         <v>168</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>79</v>
@@ -4304,11 +4074,8 @@
       <c r="I75" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J75" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A76" s="1" t="s">
         <v>268</v>
       </c>
@@ -4316,7 +4083,7 @@
         <v>169</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>80</v>
@@ -4336,11 +4103,8 @@
       <c r="I76" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J76" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A77" s="1" t="s">
         <v>269</v>
       </c>
@@ -4348,7 +4112,7 @@
         <v>170</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>81</v>
@@ -4368,11 +4132,8 @@
       <c r="I77" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J77" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A78" s="1" t="s">
         <v>270</v>
       </c>
@@ -4380,7 +4141,7 @@
         <v>171</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D78" s="1" t="s">
         <v>82</v>
@@ -4400,11 +4161,8 @@
       <c r="I78" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J78" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A79" s="1" t="s">
         <v>271</v>
       </c>
@@ -4412,7 +4170,7 @@
         <v>172</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>83</v>
@@ -4432,11 +4190,8 @@
       <c r="I79" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J79" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A80" s="1" t="s">
         <v>272</v>
       </c>
@@ -4444,7 +4199,7 @@
         <v>173</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D80" s="1" t="s">
         <v>84</v>
@@ -4464,11 +4219,8 @@
       <c r="I80" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J80" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A81" s="1" t="s">
         <v>273</v>
       </c>
@@ -4476,7 +4228,7 @@
         <v>174</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>85</v>
@@ -4496,11 +4248,8 @@
       <c r="I81" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J81" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A82" s="1" t="s">
         <v>274</v>
       </c>
@@ -4508,7 +4257,7 @@
         <v>175</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>86</v>
@@ -4528,11 +4277,8 @@
       <c r="I82" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J82" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A83" s="1" t="s">
         <v>275</v>
       </c>
@@ -4540,7 +4286,7 @@
         <v>176</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D83" s="1" t="s">
         <v>87</v>
@@ -4560,11 +4306,8 @@
       <c r="I83" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J83" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A84" s="1" t="s">
         <v>276</v>
       </c>
@@ -4572,7 +4315,7 @@
         <v>177</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D84" s="1" t="s">
         <v>88</v>
@@ -4592,11 +4335,8 @@
       <c r="I84" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J84" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A85" s="1" t="s">
         <v>277</v>
       </c>
@@ -4604,7 +4344,7 @@
         <v>178</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D85" s="1" t="s">
         <v>89</v>
@@ -4624,11 +4364,8 @@
       <c r="I85" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J85" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A86" s="1" t="s">
         <v>278</v>
       </c>
@@ -4636,7 +4373,7 @@
         <v>179</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>90</v>
@@ -4656,11 +4393,8 @@
       <c r="I86" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J86" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A87" s="1" t="s">
         <v>279</v>
       </c>
@@ -4668,7 +4402,7 @@
         <v>180</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>91</v>
@@ -4688,11 +4422,8 @@
       <c r="I87" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J87" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A88" s="1" t="s">
         <v>280</v>
       </c>
@@ -4700,7 +4431,7 @@
         <v>181</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>92</v>
@@ -4720,11 +4451,8 @@
       <c r="I88" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J88" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A89" s="1" t="s">
         <v>281</v>
       </c>
@@ -4732,7 +4460,7 @@
         <v>182</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D89" s="1" t="s">
         <v>93</v>
@@ -4752,11 +4480,8 @@
       <c r="I89" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J89" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A90" s="1" t="s">
         <v>282</v>
       </c>
@@ -4764,7 +4489,7 @@
         <v>183</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>94</v>
@@ -4784,11 +4509,8 @@
       <c r="I90" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J90" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A91" s="1" t="s">
         <v>283</v>
       </c>
@@ -4796,7 +4518,7 @@
         <v>184</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>95</v>
@@ -4816,11 +4538,8 @@
       <c r="I91" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J91" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A92" s="1" t="s">
         <v>284</v>
       </c>
@@ -4828,7 +4547,7 @@
         <v>185</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D92" s="1" t="s">
         <v>96</v>
@@ -4848,11 +4567,8 @@
       <c r="I92" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J92" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A93" s="1" t="s">
         <v>285</v>
       </c>
@@ -4860,7 +4576,7 @@
         <v>186</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>97</v>
@@ -4880,11 +4596,8 @@
       <c r="I93" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J93" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A94" s="1" t="s">
         <v>286</v>
       </c>
@@ -4892,7 +4605,7 @@
         <v>187</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>98</v>
@@ -4912,11 +4625,8 @@
       <c r="I94" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J94" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A95" s="1" t="s">
         <v>287</v>
       </c>
@@ -4924,7 +4634,7 @@
         <v>188</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>99</v>
@@ -4944,11 +4654,8 @@
       <c r="I95" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J95" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A96" s="1" t="s">
         <v>288</v>
       </c>
@@ -4956,7 +4663,7 @@
         <v>189</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>100</v>
@@ -4976,11 +4683,8 @@
       <c r="I96" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J96" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A97" s="1" t="s">
         <v>289</v>
       </c>
@@ -4988,7 +4692,7 @@
         <v>190</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>101</v>
@@ -5008,11 +4712,8 @@
       <c r="I97" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J97" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A98" s="1" t="s">
         <v>290</v>
       </c>
@@ -5020,7 +4721,7 @@
         <v>191</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="D98" s="1" t="s">
         <v>102</v>
@@ -5040,11 +4741,8 @@
       <c r="I98" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J98" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A99" s="1" t="s">
         <v>291</v>
       </c>
@@ -5052,7 +4750,7 @@
         <v>192</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="D99" s="1" t="s">
         <v>103</v>
@@ -5072,11 +4770,8 @@
       <c r="I99" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J99" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A100" s="1" t="s">
         <v>292</v>
       </c>
@@ -5084,7 +4779,7 @@
         <v>193</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>104</v>
@@ -5104,11 +4799,8 @@
       <c r="I100" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J100" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A101" s="1" t="s">
         <v>293</v>
       </c>
@@ -5116,7 +4808,7 @@
         <v>293</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="D101" s="1" t="s">
         <v>105</v>
@@ -5136,11 +4828,8 @@
       <c r="I101" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J101" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A102" s="1" t="s">
         <v>294</v>
       </c>
@@ -5148,7 +4837,7 @@
         <v>294</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D102" s="1" t="s">
         <v>106</v>
@@ -5168,11 +4857,8 @@
       <c r="I102" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J102" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A103" s="1" t="s">
         <v>295</v>
       </c>
@@ -5180,7 +4866,7 @@
         <v>295</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="D103" s="1" t="s">
         <v>107</v>
@@ -5200,11 +4886,8 @@
       <c r="I103" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J103" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A104" s="1" t="s">
         <v>296</v>
       </c>
@@ -5212,7 +4895,7 @@
         <v>296</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D104" s="1" t="s">
         <v>108</v>
@@ -5232,11 +4915,8 @@
       <c r="I104" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J104" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A105" s="1" t="s">
         <v>297</v>
       </c>
@@ -5244,7 +4924,7 @@
         <v>297</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>109</v>
@@ -5264,11 +4944,8 @@
       <c r="I105" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J105" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A106" s="1" t="s">
         <v>298</v>
       </c>
@@ -5276,7 +4953,7 @@
         <v>298</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="D106" s="1" t="s">
         <v>110</v>
@@ -5296,11 +4973,8 @@
       <c r="I106" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J106" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A107" s="1" t="s">
         <v>299</v>
       </c>
@@ -5308,7 +4982,7 @@
         <v>299</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="D107" s="1" t="s">
         <v>76</v>
@@ -5328,11 +5002,8 @@
       <c r="I107" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J107" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A108" s="1" t="s">
         <v>300</v>
       </c>
@@ -5340,7 +5011,7 @@
         <v>300</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="D108" s="1" t="s">
         <v>77</v>
@@ -5360,11 +5031,8 @@
       <c r="I108" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J108" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A109" s="1" t="s">
         <v>301</v>
       </c>
@@ -5372,7 +5040,7 @@
         <v>301</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="D109" s="1" t="s">
         <v>78</v>
@@ -5392,11 +5060,8 @@
       <c r="I109" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J109" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A110" s="1" t="s">
         <v>302</v>
       </c>
@@ -5404,7 +5069,7 @@
         <v>302</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D110" s="1" t="s">
         <v>79</v>
@@ -5424,11 +5089,8 @@
       <c r="I110" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J110" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A111" s="1" t="s">
         <v>303</v>
       </c>
@@ -5436,7 +5098,7 @@
         <v>303</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="D111" s="1" t="s">
         <v>80</v>
@@ -5456,11 +5118,8 @@
       <c r="I111" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J111" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A112" s="1" t="s">
         <v>304</v>
       </c>
@@ -5468,7 +5127,7 @@
         <v>304</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="D112" s="1" t="s">
         <v>81</v>
@@ -5488,11 +5147,8 @@
       <c r="I112" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J112" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A113" s="1" t="s">
         <v>305</v>
       </c>
@@ -5500,7 +5156,7 @@
         <v>305</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="D113" s="1" t="s">
         <v>82</v>
@@ -5520,11 +5176,8 @@
       <c r="I113" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J113" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A114" s="1" t="s">
         <v>306</v>
       </c>
@@ -5532,7 +5185,7 @@
         <v>306</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="D114" s="1" t="s">
         <v>83</v>
@@ -5552,11 +5205,8 @@
       <c r="I114" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J114" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A115" s="1" t="s">
         <v>307</v>
       </c>
@@ -5564,7 +5214,7 @@
         <v>307</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="D115" s="1" t="s">
         <v>84</v>
@@ -5584,11 +5234,8 @@
       <c r="I115" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J115" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A116" s="1" t="s">
         <v>308</v>
       </c>
@@ -5596,7 +5243,7 @@
         <v>308</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="D116" s="1" t="s">
         <v>85</v>
@@ -5616,11 +5263,8 @@
       <c r="I116" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J116" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A117" s="1" t="s">
         <v>309</v>
       </c>
@@ -5628,7 +5272,7 @@
         <v>309</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="D117" s="1" t="s">
         <v>86</v>
@@ -5648,11 +5292,8 @@
       <c r="I117" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J117" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A118" s="1" t="s">
         <v>310</v>
       </c>
@@ -5660,7 +5301,7 @@
         <v>310</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D118" s="1" t="s">
         <v>87</v>
@@ -5680,11 +5321,8 @@
       <c r="I118" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J118" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A119" s="1" t="s">
         <v>311</v>
       </c>
@@ -5692,7 +5330,7 @@
         <v>311</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D119" s="1" t="s">
         <v>88</v>
@@ -5712,11 +5350,8 @@
       <c r="I119" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J119" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A120" s="1" t="s">
         <v>312</v>
       </c>
@@ -5724,7 +5359,7 @@
         <v>312</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D120" s="1" t="s">
         <v>89</v>
@@ -5744,11 +5379,8 @@
       <c r="I120" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J120" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A121" s="1" t="s">
         <v>313</v>
       </c>
@@ -5756,7 +5388,7 @@
         <v>313</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="D121" s="1" t="s">
         <v>90</v>
@@ -5776,11 +5408,8 @@
       <c r="I121" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J121" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A122" s="1" t="s">
         <v>314</v>
       </c>
@@ -5788,7 +5417,7 @@
         <v>314</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D122" s="1" t="s">
         <v>91</v>
@@ -5808,11 +5437,8 @@
       <c r="I122" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J122" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A123" s="1" t="s">
         <v>315</v>
       </c>
@@ -5820,7 +5446,7 @@
         <v>315</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="D123" s="1" t="s">
         <v>92</v>
@@ -5840,11 +5466,8 @@
       <c r="I123" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J123" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A124" s="1" t="s">
         <v>316</v>
       </c>
@@ -5852,7 +5475,7 @@
         <v>316</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="D124" s="1" t="s">
         <v>93</v>
@@ -5872,11 +5495,8 @@
       <c r="I124" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J124" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A125" s="1" t="s">
         <v>317</v>
       </c>
@@ -5884,7 +5504,7 @@
         <v>317</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="D125" s="1" t="s">
         <v>94</v>
@@ -5904,11 +5524,8 @@
       <c r="I125" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J125" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A126" s="1" t="s">
         <v>318</v>
       </c>
@@ -5916,7 +5533,7 @@
         <v>318</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="D126" s="1" t="s">
         <v>95</v>
@@ -5936,11 +5553,8 @@
       <c r="I126" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J126" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A127" s="1" t="s">
         <v>319</v>
       </c>
@@ -5948,7 +5562,7 @@
         <v>319</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D127" s="1" t="s">
         <v>96</v>
@@ -5968,11 +5582,8 @@
       <c r="I127" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J127" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A128" s="1" t="s">
         <v>320</v>
       </c>
@@ -5980,7 +5591,7 @@
         <v>320</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="D128" s="1" t="s">
         <v>97</v>
@@ -6000,11 +5611,8 @@
       <c r="I128" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J128" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A129" s="1" t="s">
         <v>321</v>
       </c>
@@ -6012,7 +5620,7 @@
         <v>321</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="D129" s="1" t="s">
         <v>98</v>
@@ -6032,11 +5640,8 @@
       <c r="I129" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J129" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A130" s="1" t="s">
         <v>322</v>
       </c>
@@ -6044,7 +5649,7 @@
         <v>322</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="D130" s="1" t="s">
         <v>99</v>
@@ -6064,11 +5669,8 @@
       <c r="I130" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J130" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A131" s="1" t="s">
         <v>323</v>
       </c>
@@ -6076,7 +5678,7 @@
         <v>323</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="D131" s="1" t="s">
         <v>100</v>
@@ -6096,11 +5698,8 @@
       <c r="I131" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J131" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A132" s="1" t="s">
         <v>324</v>
       </c>
@@ -6108,7 +5707,7 @@
         <v>324</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="D132" s="1" t="s">
         <v>101</v>
@@ -6128,11 +5727,8 @@
       <c r="I132" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J132" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A133" s="1" t="s">
         <v>325</v>
       </c>
@@ -6140,7 +5736,7 @@
         <v>325</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>102</v>
@@ -6160,11 +5756,8 @@
       <c r="I133" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J133" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A134" s="1" t="s">
         <v>326</v>
       </c>
@@ -6172,7 +5765,7 @@
         <v>326</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D134" s="1" t="s">
         <v>103</v>
@@ -6192,11 +5785,8 @@
       <c r="I134" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J134" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A135" s="1" t="s">
         <v>327</v>
       </c>
@@ -6204,7 +5794,7 @@
         <v>327</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D135" s="1" t="s">
         <v>104</v>
@@ -6224,11 +5814,8 @@
       <c r="I135" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J135" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A136" s="1" t="s">
         <v>328</v>
       </c>
@@ -6236,7 +5823,7 @@
         <v>328</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D136" s="1" t="s">
         <v>105</v>
@@ -6256,11 +5843,8 @@
       <c r="I136" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J136" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A137" s="1" t="s">
         <v>329</v>
       </c>
@@ -6268,7 +5852,7 @@
         <v>329</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D137" s="1" t="s">
         <v>106</v>
@@ -6288,11 +5872,8 @@
       <c r="I137" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J137" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A138" s="1" t="s">
         <v>330</v>
       </c>
@@ -6300,7 +5881,7 @@
         <v>330</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="D138" s="1" t="s">
         <v>107</v>
@@ -6320,11 +5901,8 @@
       <c r="I138" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J138" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A139" s="1" t="s">
         <v>331</v>
       </c>
@@ -6332,7 +5910,7 @@
         <v>331</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="D139" s="1" t="s">
         <v>108</v>
@@ -6352,11 +5930,8 @@
       <c r="I139" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J139" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A140" s="1" t="s">
         <v>332</v>
       </c>
@@ -6364,7 +5939,7 @@
         <v>332</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="D140" s="1" t="s">
         <v>109</v>
@@ -6384,11 +5959,8 @@
       <c r="I140" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J140" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A141" s="1" t="s">
         <v>333</v>
       </c>
@@ -6396,7 +5968,7 @@
         <v>333</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="D141" s="1" t="s">
         <v>110</v>
@@ -6416,161 +5988,19 @@
       <c r="I141" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J141" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.15">
       <c r="C142" s="2"/>
     </row>
-    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="145" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="146" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="147" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="148" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="149" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="150" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="151" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="152" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="153" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="154" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="155" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="156" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="157" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="158" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="159" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="160" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="161" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="162" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="163" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="164" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="165" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="166" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="167" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="168" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="169" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="170" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="171" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="172" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="173" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="174" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="175" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="176" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="177" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="178" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="179" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="180" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="181" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="182" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="183" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="184" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="185" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="186" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="187" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="188" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="189" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="190" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="191" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="192" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="193" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="194" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="195" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="196" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="197" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="198" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="199" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="200" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="201" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="202" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="203" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="204" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="205" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="206" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="207" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="208" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="209" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="210" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="211" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="212" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="213" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="214" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="215" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="216" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="217" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="218" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="219" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="220" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="221" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="222" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="223" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="224" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="225" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="226" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="227" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="228" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="229" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="230" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="231" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="232" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="233" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="234" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="235" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="236" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="237" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="238" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="239" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="240" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="241" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="242" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="243" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="244" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="245" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="246" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="247" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="248" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="249" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="250" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="251" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="252" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="253" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="254" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="255" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="256" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="257" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="258" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="259" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="260" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="261" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="262" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="263" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="264" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="265" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="266" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="267" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="268" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="269" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="270" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="271" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="272" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="273" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="274" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="275" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="276" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="277" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="278" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="279" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="280" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="281" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.15">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A282" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C282" s="1" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D282" s="1" t="s">
         <v>335</v>
@@ -6584,19 +6014,16 @@
       <c r="I282" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J282" s="1" t="s">
+    </row>
+    <row r="283" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A283" s="1" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A283" s="1" t="s">
-        <v>339</v>
-      </c>
       <c r="B283" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C283" s="1" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D283" s="1" t="s">
         <v>335</v>
@@ -6610,19 +6037,16 @@
       <c r="I283" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J283" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="284" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A284" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C284" s="1" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D284" s="1" t="s">
         <v>335</v>
@@ -6636,19 +6060,16 @@
       <c r="I284" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J284" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="285" spans="1:10" x14ac:dyDescent="0.15">
+    </row>
+    <row r="285" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A285" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C285" s="1" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D285" s="1" t="s">
         <v>335</v>
@@ -6662,22 +6083,8 @@
       <c r="I285" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J285" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="286" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="287" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="288" spans="1:10" hidden="1" x14ac:dyDescent="0.15"/>
-    <row r="289" hidden="1" x14ac:dyDescent="0.15"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M430" xr:uid="{67D76F6C-B8F9-3044-BD3D-2174C4F373AB}">
-    <filterColumn colId="9">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>